<commit_message>
WIP: payment structure analysis, return to NaN Payment Type
</commit_message>
<xml_diff>
--- a/reports/data_dictionary _processed.xlsx
+++ b/reports/data_dictionary _processed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Final Project Python\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E2DE63-F0EE-4EC5-8C21-222A3754A326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC10D85-EA33-49F6-8FE5-F88224046327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-2610" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Deals" sheetId="1" r:id="rId1"/>
     <sheet name="Calls" sheetId="2" r:id="rId2"/>
     <sheet name="Spend" sheetId="3" r:id="rId3"/>
+    <sheet name="Contacts" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="176">
   <si>
     <t>Column</t>
   </si>
@@ -80,9 +81,6 @@
     <t>Имя менеджера-владельца сделки</t>
   </si>
   <si>
-    <t>не удаляем</t>
-  </si>
-  <si>
     <t>Closing Date</t>
   </si>
   <si>
@@ -92,9 +90,6 @@
     <t>Дата завершения работы по сделке (закрытия — успешного или с потерей)</t>
   </si>
   <si>
-    <t>дата в диапазоне периода данных</t>
-  </si>
-  <si>
     <t>Quality</t>
   </si>
   <si>
@@ -125,9 +120,6 @@
     <t>22 уникальных значения</t>
   </si>
   <si>
-    <t>NaN сохраняем (для не-Lost сделок)</t>
-  </si>
-  <si>
     <t>Page</t>
   </si>
   <si>
@@ -158,9 +150,6 @@
     <t>неотрицательная длительность</t>
   </si>
   <si>
-    <t>NaN сохраняем; единичные SLA &gt; 30 дней отмечаем как аномалии</t>
-  </si>
-  <si>
     <t>Content</t>
   </si>
   <si>
@@ -185,9 +174,6 @@
     <t>13 значений: Facebook Ads, Google Ads, Organic, Test и др.</t>
   </si>
   <si>
-    <t>NaN сохраняем (2 случая)</t>
-  </si>
-  <si>
     <t>Payment Type</t>
   </si>
   <si>
@@ -239,9 +225,6 @@
     <t>0–11 (целое число)</t>
   </si>
   <si>
-    <t>NaN сохраняем (для неактивных учеников)</t>
-  </si>
-  <si>
     <t>Initial Amount Paid</t>
   </si>
   <si>
@@ -254,18 +237,12 @@
     <t>0–11500</t>
   </si>
   <si>
-    <t>NaN сохраняем; нормализация европейского формата € X.XXX,YY</t>
-  </si>
-  <si>
     <t>Offer Total Amount</t>
   </si>
   <si>
     <t>Полная стоимость обучения по договору (сколько клиент заплатит, если доучится до конца и внесёт все платежи)</t>
   </si>
   <si>
-    <t>NaN сохраняем; нормализация европейского формата</t>
-  </si>
-  <si>
     <t>Contact Name</t>
   </si>
   <si>
@@ -275,9 +252,6 @@
     <t>19-значное число как строка</t>
   </si>
   <si>
-    <t>NaN сохраняем (63 случая)</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
@@ -287,9 +261,6 @@
     <t>название города на немецком</t>
   </si>
   <si>
-    <t>"-" (348 случаев) → NaN; NaN сохраняем</t>
-  </si>
-  <si>
     <t>Level of Deutsch</t>
   </si>
   <si>
@@ -299,18 +270,12 @@
     <t>A1, A2, B1, B2, C1, C2</t>
   </si>
   <si>
-    <t>Нормализация: regex-экстрактор букв и цифр; кириллица → латиница; верхний регистр. Свободный текст без явного уровня → NaN</t>
-  </si>
-  <si>
     <t>Stage_Group</t>
   </si>
   <si>
     <t>[Производная] Группировка Stage для анализа воронки</t>
   </si>
   <si>
-    <t>Won, Lost, In Progress, Free</t>
-  </si>
-  <si>
     <t>создаётся в чистке через mapping</t>
   </si>
   <si>
@@ -356,9 +321,6 @@
     <t>Имя менеджера, совершившего/принявшего звонок</t>
   </si>
   <si>
-    <t>33 уникальных значения (включая менеджеров не из Deals)</t>
-  </si>
-  <si>
     <t>CONTACTID</t>
   </si>
   <si>
@@ -381,12 +343,6 @@
   </si>
   <si>
     <t>Продолжительность звонка в секундах</t>
-  </si>
-  <si>
-    <t>≥ 0; 22% звонков = 0 (не дозвонился до гудка / сбросил)</t>
-  </si>
-  <si>
-    <t>NaN сохраняем (83 случая)</t>
   </si>
   <si>
     <t>Call Status</t>
@@ -611,8 +567,88 @@
         <scheme val="minor"/>
       </rPr>
       <t>.
-- также отдельно флаг is_won_confirmed - где сумма больше 0 и статус Pdone</t>
+- также отдельно флаг is_won_confirmed - где сумма больше 1 и статус Payment done (больше 1 тк есть условный курс введения в айти чтоб его исключить)</t>
     </r>
+  </si>
+  <si>
+    <t>Рассматриваем только по статусу Lost -  без статуса клиент не считается Lost. (Также поле используется для причины переноса на след поток Next stream и для исторических записях о трудностях).</t>
+  </si>
+  <si>
+    <t>is_won_confirmed</t>
+  </si>
+  <si>
+    <t>is_main_product</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> is_closing_date_anomaly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При One Payment есть значения, которые не совпадают польностью с полной стоимостью курса. Поэтому оставим как есть - принимаю что значение указывает на выбранную клиентом форму договора, а не фактическую полноту оплаты на момент выгрузки. Несовпадающие суммы - это предоплата. </t>
+  </si>
+  <si>
+    <t>SLA &gt; 30 дней: 91
+Доля аномалий: 0.59%</t>
+  </si>
+  <si>
+    <t>нормализация европейского формата € X.XXX,YY в число без значка евро</t>
+  </si>
+  <si>
+    <t>NaN сохраняем (61 случай)</t>
+  </si>
+  <si>
+    <t>"-" (348 случаев) заменили на NaN;</t>
+  </si>
+  <si>
+    <t>Нормализация: regex-экстрактор букв и цифр; кириллица → латиница; верхний регистр. Свободный текст без явного уровня заменили на Nan</t>
+  </si>
+  <si>
+    <t>Won, Lost, In Progress</t>
+  </si>
+  <si>
+    <t>создаётся в чистке через mapping, Free Education в Won</t>
+  </si>
+  <si>
+    <t>видимо заполняется автоматически</t>
+  </si>
+  <si>
+    <t xml:space="preserve">True для сделок, где Stage = 'Payment Done' 
+И Initial Amount Paid &gt; 1. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Флаг основного продукта. </t>
+  </si>
+  <si>
+    <t>Stage_Group = 'Won' включает все 859 Payment Done, is_won_confirmed = True — только 839 с подтверждённой оплатой.</t>
+  </si>
+  <si>
+    <t>True для:Web Developer, Digital Marketing, UX/UI Design.
+False для Find yourself in IT, Data Analytics и сделок без указанного продукта.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Флаг хронологической аномалии. </t>
+  </si>
+  <si>
+    <t>True для сделок, где Closing Date раньше 
+Created Time (физически невозможно). 44 случая — вероятно опечатки 
+менеджеров при ручном вводе даты. Сами сделки сохранены в датасете, исключаются только из расчёта времени до закрытия.</t>
+  </si>
+  <si>
+    <t>33 уникальных Call Owner против 27 в Deals — часть менеджеров работает только 
+со звонками, не ведя сделки (junior-уровень / call-center / уволенные сотрудники, 
+точная природа требует уточнения у заказчика).</t>
+  </si>
+  <si>
+    <t>от 0 до 7625 секунд (около 2 часов)</t>
+  </si>
+  <si>
+    <t>дата в диапазоне периода данных 2023-06-30 08:43:00
+2024-06-21 15:31:00</t>
+  </si>
+  <si>
+    <t>Contact Owner Name</t>
+  </si>
+  <si>
+    <t>Modified Time</t>
   </si>
 </sst>
 </file>
@@ -684,7 +720,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -708,6 +744,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -723,6 +760,196 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2139315</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>107632</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>382905</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40BEAABD-2293-4DDB-9745-1385F6A05E36}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2139315" y="107632"/>
+          <a:ext cx="5873115" cy="1082993"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>Таблица </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Contacts </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>не использовалась в анализе. Содержит только технические </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>поля (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Id, Contact Owner Name, Created Time, Modified Time) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>без атрибутов </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>контактов (имя, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>email, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>телефон, демография). Информация о контакте, </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>необходимая для анализа (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>City, Level of Deutsch, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>и т.д.), содержится </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>напрямую в </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Deals.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>544830</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="184731" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8732F10D-1F43-4B30-A22B-8D506715939F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12441555" y="5440680"/>
+          <a:ext cx="184731" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1010,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="4" customWidth="1"/>
@@ -1061,7 +1288,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1081,10 +1308,10 @@
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="E3" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1095,19 +1322,19 @@
     </row>
     <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="G4">
         <v>6948</v>
@@ -1118,19 +1345,19 @@
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="G5">
         <v>2256</v>
@@ -1139,44 +1366,44 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>29</v>
+        <v>152</v>
       </c>
       <c r="G7">
         <v>5469</v>
@@ -1186,43 +1413,43 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G9">
         <v>5526</v>
@@ -1232,20 +1459,20 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>40</v>
+        <v>157</v>
       </c>
       <c r="G10">
         <v>6060</v>
@@ -1255,20 +1482,17 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>41</v>
+      <c r="A11" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="G11">
         <v>7446</v>
@@ -1278,20 +1502,17 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>44</v>
+      <c r="A12" s="7" t="s">
+        <v>40</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="G12">
         <v>9139</v>
@@ -1301,43 +1522,40 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>25</v>
+        <v>156</v>
       </c>
       <c r="G14">
         <v>21097</v>
@@ -1348,19 +1566,19 @@
     </row>
     <row r="15" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="G15">
         <v>18001</v>
@@ -1370,20 +1588,17 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>55</v>
+      <c r="A16" s="7" t="s">
+        <v>50</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="G16">
         <v>18294</v>
@@ -1394,42 +1609,39 @@
     </row>
     <row r="17" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="G18">
         <v>18006</v>
@@ -1438,21 +1650,18 @@
         <v>83.4</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>64</v>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>59</v>
       </c>
       <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="G19">
         <v>20753</v>
@@ -1462,20 +1671,20 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>68</v>
+      <c r="A20" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="G20">
         <v>17428</v>
@@ -1485,20 +1694,17 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>73</v>
+      <c r="A21" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G21">
         <v>17408</v>
@@ -1508,20 +1714,20 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>76</v>
+      <c r="A22" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="G22">
         <v>61</v>
@@ -1531,20 +1737,20 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>80</v>
+      <c r="A23" s="7" t="s">
+        <v>71</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>83</v>
+        <v>160</v>
       </c>
       <c r="G23">
         <v>19430</v>
@@ -1553,21 +1759,21 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>84</v>
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>87</v>
+        <v>161</v>
       </c>
       <c r="G24">
         <v>20400</v>
@@ -1577,20 +1783,20 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
-        <v>88</v>
+      <c r="A25" s="7" t="s">
+        <v>77</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>90</v>
+        <v>162</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>91</v>
+        <v>163</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -1600,20 +1806,20 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>92</v>
+      <c r="A26" s="7" t="s">
+        <v>80</v>
       </c>
       <c r="B26" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -1623,26 +1829,77 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>97</v>
+      <c r="A27" s="7" t="s">
+        <v>85</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
         <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="B28" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1655,51 +1912,53 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="57.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="28.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
+      <c r="C2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1708,24 +1967,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>102</v>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1734,24 +1987,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>104</v>
+    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>92</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
+      <c r="C4" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1760,24 +2007,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>107</v>
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>94</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" t="s">
-        <v>109</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
+      <c r="C5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="G5">
         <v>3933</v>
@@ -1786,50 +2030,41 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>110</v>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>97</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="C6" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E7" t="s">
-        <v>116</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
+      <c r="D7" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="G7">
         <v>83</v>
@@ -1838,24 +2073,18 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>117</v>
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>102</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E8" t="s">
-        <v>101</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
+      <c r="C8" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1864,24 +2093,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>120</v>
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>105</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" t="s">
-        <v>123</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
+      <c r="C9" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="G9">
         <v>8999</v>
@@ -1891,23 +2117,20 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>124</v>
+      <c r="A10" s="9" t="s">
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" t="s">
-        <v>125</v>
-      </c>
-      <c r="D10" t="s">
-        <v>126</v>
-      </c>
-      <c r="E10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
+        <v>56</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="G10">
         <v>8999</v>
@@ -1916,24 +2139,21 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>128</v>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" t="s">
-        <v>14</v>
+        <v>81</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1944,6 +2164,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1951,51 +2172,56 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="42.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="48.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>131</v>
+      <c r="A2" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2004,24 +2230,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>46</v>
+    <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
+      <c r="C3" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2030,24 +2253,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>33</v>
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
+      <c r="C4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="G4">
         <v>5077</v>
@@ -2057,23 +2277,17 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>139</v>
+      <c r="A5" s="9" t="s">
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" t="s">
-        <v>141</v>
-      </c>
-      <c r="D5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
+        <v>125</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2083,23 +2297,17 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>143</v>
+      <c r="A6" s="9" t="s">
+        <v>128</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
+        <v>63</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -2108,24 +2316,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>146</v>
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" t="s">
-        <v>147</v>
-      </c>
-      <c r="D7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E7" t="s">
-        <v>101</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
+        <v>125</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -2134,24 +2336,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>149</v>
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>134</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D8" t="s">
-        <v>151</v>
-      </c>
-      <c r="E8" t="s">
-        <v>152</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
+      <c r="C8" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="G8">
         <v>5911</v>
@@ -2161,23 +2360,20 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>153</v>
+      <c r="A9" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
-        <v>154</v>
-      </c>
-      <c r="D9" t="s">
-        <v>155</v>
-      </c>
-      <c r="E9" t="s">
-        <v>156</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
+      <c r="C9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="G9">
         <v>5911</v>
@@ -2189,4 +2385,41 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A414200-B27D-4927-AA5E-604EABD9396E}">
+  <dimension ref="A2:A6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: restore Payment Type for 478 Won deals using financial logic (Recurring/One Payment ratios)
</commit_message>
<xml_diff>
--- a/reports/data_dictionary _processed.xlsx
+++ b/reports/data_dictionary _processed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Final Project Python\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC10D85-EA33-49F6-8FE5-F88224046327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96EEFEFB-6ADF-4C80-B8E7-B1979A102453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-2610" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="177">
   <si>
     <t>Column</t>
   </si>
@@ -649,6 +649,14 @@
   </si>
   <si>
     <t>Modified Time</t>
+  </si>
+  <si>
+    <t>Всего Won Confirmed: 839
+С Payment Type: 360 
+Без Payment Type (NaN): 479
+Заполнено как Recurring Payments: 462
+Заполнено как One Payment: 16
+Осталось NaN среди Won Confirmed: 1</t>
   </si>
 </sst>
 </file>
@@ -1541,7 +1549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
@@ -1556,6 +1564,9 @@
       </c>
       <c r="E14" s="1" t="s">
         <v>156</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="G14">
         <v>21097</v>

</xml_diff>